<commit_message>
added 4A and updated previous files
</commit_message>
<xml_diff>
--- a/Lee_Ex3A_tables.xlsx
+++ b/Lee_Ex3A_tables.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leech\Documents\DATA_Labs\W2_Workshop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{514E36D5-267F-4831-81BC-244C12944B31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA54DC93-7292-4179-9274-096F614DD191}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="12860" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="11290" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dog Owner" sheetId="1" r:id="rId1"/>
     <sheet name="Dog" sheetId="2" r:id="rId2"/>
-    <sheet name="Walk" sheetId="3" r:id="rId3"/>
-    <sheet name="Payment" sheetId="4" r:id="rId4"/>
+    <sheet name="Payment" sheetId="4" r:id="rId3"/>
+    <sheet name="Walk" sheetId="3" r:id="rId4"/>
     <sheet name="Walker" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="162913"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="33">
   <si>
     <t>first_name</t>
   </si>
@@ -122,6 +122,12 @@
   </si>
   <si>
     <t>emergency_contact_phone</t>
+  </si>
+  <si>
+    <t>5,2</t>
+  </si>
+  <si>
+    <t>10,2</t>
   </si>
 </sst>
 </file>
@@ -169,10 +175,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -453,55 +460,89 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="23.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="23" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="23.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="3"/>
+      <c r="I1" s="3"/>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B4">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B5">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B6">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B7">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B8">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>30</v>
+      </c>
+      <c r="B9">
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -511,53 +552,73 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67516B79-9633-47B0-AA1B-8B32A6A62E7D}">
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.7265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="3"/>
+      <c r="I1" s="3"/>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B4">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B6">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B7" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -568,56 +629,54 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09C74533-0349-417B-AEAD-CD65EB081889}">
-  <dimension ref="A1:A9"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3AAC0221-239D-4E8B-ABD1-17A5C45843E4}">
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+        <v>22</v>
+      </c>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+        <v>25</v>
+      </c>
+      <c r="B5">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -626,41 +685,62 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3AAC0221-239D-4E8B-ABD1-17A5C45843E4}">
-  <dimension ref="A1:A6"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09C74533-0349-417B-AEAD-CD65EB081889}">
+  <dimension ref="A1:B9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="15.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>26</v>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>21</v>
+      </c>
+      <c r="B9">
+        <v>225</v>
       </c>
     </row>
   </sheetData>
@@ -670,37 +750,52 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{718233ED-B443-4B7A-A17D-8C42C3917532}">
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="9.81640625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B4">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B5">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>3</v>
+      </c>
+      <c r="B6">
+        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>